<commit_message>
Actualizacion de la interface visual de SCMBD. Filtros Catalogo de Relacion Usuario Operaciones.
</commit_message>
<xml_diff>
--- a/SCMBD/Documentos/Pantalla relUsuaioOPeracion.xlsx
+++ b/SCMBD/Documentos/Pantalla relUsuaioOPeracion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Desarrollos\DesarrollosVisual\SCMBD\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{598CE88B-FDDD-4A31-AC62-8ED457E0C73C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D74328FF-9B49-4A2E-B1BA-073AC686FD73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{360F5ACE-DCE3-4C8C-978F-C702FC208524}"/>
   </bookViews>
@@ -74,10 +74,10 @@
     <t>Inactivo</t>
   </si>
   <si>
-    <t>Columna1</t>
-  </si>
-  <si>
     <t>Estatus Relacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     _</t>
   </si>
 </sst>
 </file>
@@ -636,7 +636,7 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{8E3E1C45-7FC7-4C92-AF46-B18367E8348B}" name="Operacion"/>
     <tableColumn id="2" xr3:uid="{45D0A14E-AAB6-4A30-B790-A6B86EF3EAE6}" name="Autorizacion"/>
-    <tableColumn id="4" xr3:uid="{1BB1BE76-3B15-4155-958A-3D96F4591D90}" name="Columna1"/>
+    <tableColumn id="4" xr3:uid="{1BB1BE76-3B15-4155-958A-3D96F4591D90}" name="     _"/>
     <tableColumn id="3" xr3:uid="{1BEB4325-82FD-4EF7-88B5-1B02BE06CADE}" name="Estatus Relacion"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -977,10 +977,10 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
         <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">

</xml_diff>